<commit_message>
Records: Open Items v0.7 adds OI-21 (DEC-003's VPS never existed); AI Usage Register v0.13 row 59
Open Items v0.7: OI-21 at row 25 and the B2 version note; the closing note moves to row 26 with
its merge. AI Usage Register v0.13: row 59 (B59:I59). No version bump: both workbooks are already
new in this PR, and Open Items v0.6 took OI-20 the same way.

Compared cell by cell against f56cc04: only those cells changed, plus row heights, the saved view
and Excel's save metadata.
</commit_message>
<xml_diff>
--- a/docs/AI-Usage/AI Usage Register/AI Usage Register v0.13.xlsx
+++ b/docs/AI-Usage/AI Usage Register/AI Usage Register v0.13.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huawei\Desktop\SEN381\Ticketing-System\docs\AI-Usage\AI Usage Register\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35EF64D2-7160-4985-9618-BE3571806CAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A78C0EAD-A1F7-49C1-AB5A-153B36A239C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13200" yWindow="0" windowWidth="13543" windowHeight="17829" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13286" yWindow="0" windowWidth="13543" windowHeight="17914" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AI Usage Register" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="269">
   <si>
     <t>AI Usage Register</t>
   </si>
@@ -921,6 +921,24 @@
   </si>
   <si>
     <t>One. The manifest had been on dev since PR #49 (29/09/2026) and passed every required check: no gate inspects content inside images or PDFs. Raised as OI-20 rather than left implicit</t>
+  </si>
+  <si>
+    <t>TD-004 index provisioning: privilege probe, provisioning script, tests, negative verifications NV-83 to NV-90, first live check-only run (L1), PR #98; OI-21 (DEC-003 assumed a VPS that never existed), PR #96</t>
+  </si>
+  <si>
+    <t>Designed and wrote a privilege probe that ran on a throwaway database (ccprobe) on the Atlas test cluster. It showed that createIndex alone builds an index on an absent collection, so createCollection need not be granted, and that a TTL change is refused with error 85. Built the provisioning script (scripts/atlas/provision-indexes.js, indexComparison.js, declaredIndexes.js, scripts/lib/clusterMarkers.js) with a command allow-list, a server-reported privilege check and a --check-only mode. Wrote 19 tests (suite 167 → 186 pass, 8 pre-existing skips) and eight sabotage negative verifications (NV-83 to NV-90, all caught). Ran L1 check-only against the test cluster: 20 of 21 declared indexes missing, including all unique indexes (DEF-014, DEF-015, DEF-017), five declared collections absent, sessions TTL 1800 s. Drafted the evidence records, the PR #98 description and the OI-21 row.</t>
+  </si>
+  <si>
+    <t>Expected results were written before every run. I created and removed the Atlas probe and provisioner roles and users myself, and checked each role’s grants against the screen (least privilege: 10 named collections, no wildcard). The AI reproduced the implementer’s claims independently: tests, lint, guards refusing before connecting, and sabotage NV-83 re-run with matching file hashes. I checked that NV-83 to NV-90 were free with git grep across all remote branches, with an NV-82 control. OI-21 was checked across all 36 branches, including text inside Office files, with OI-20 and OI-99 controls. Gitleaks 8.18.4 found no new findings. Workbook edits were compared cell by cell against f56cc04 before commit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accepted the script, tests and records. Overruled provisioning before merge: the credential was deleted and provisioning deferred until PR #98 is reviewed. Deferred dropping the test civicconnect database (D4) until both teammates agree. </t>
+  </si>
+  <si>
+    <t>On the first full run, the implementer got 3 test failures and re-ran without capturing the test names. Recorded as a gap, not re-run to green. A Defect Register row is pending.
+I reported the cleanup times in SAST where UTC was asked, twice. The AI detected and converted them, and the records state the conversion.
+The AI’s run commands wrote output to a local AI scratchpad path, which risked an AI-local path entering committed evidence. Caught before commit; the L1 record uses a placeholder.
+The AI repeated an error from my project notes, attributing “the VPS the team already has” to DEC-003 instead of DEC-002. Caught by the AI when reading the documents before drafting OI-21.</t>
   </si>
 </sst>
 </file>
@@ -2961,15 +2979,31 @@
         <v>263</v>
       </c>
     </row>
-    <row r="59" spans="2:9">
-      <c r="B59" s="12"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="8"/>
-      <c r="F59" s="8"/>
-      <c r="G59" s="8"/>
-      <c r="H59" s="8"/>
-      <c r="I59" s="8"/>
+    <row r="59" spans="2:9" ht="276.89999999999998">
+      <c r="B59" s="12">
+        <v>46308</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="F59" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="G59" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="H59" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="I59" s="8" t="s">
+        <v>268</v>
+      </c>
     </row>
     <row r="60" spans="2:9">
       <c r="B60" s="12"/>

</xml_diff>